<commit_message>
Clarify report input workflow
</commit_message>
<xml_diff>
--- a/03_운영시트_템플릿/모먼트인사이트_운영시트_템플릿.xlsx
+++ b/03_운영시트_템플릿/모먼트인사이트_운영시트_템플릿.xlsx
@@ -2,15 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="처음_사용법" sheetId="1" r:id="R2c7a1b9ac3b74518"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="월간_매출입력" sheetId="2" r:id="R2174afa19abb45f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="네이버_일별입력" sheetId="3" r:id="Rc8cc2cd42ba548d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="쿠팡_일별입력" sheetId="4" r:id="R6db909d06af541f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보고서_목록" sheetId="5" r:id="R2dd68abb71df4c62"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="일정표" sheetId="6" r:id="R90ec35bdcd9a45e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="인사이트_액션플랜" sheetId="7" r:id="Re1a87c0e9aa14c9b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="운영_대시보드" sheetId="8" r:id="Rf007a8d38a92424c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="공개규칙" sheetId="9" r:id="R950cf343d1fe4441"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="처음_사용법" sheetId="1" r:id="R62508739f8a84892"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="월간_매출입력" sheetId="2" r:id="R24c7561897e24600"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="네이버_일별입력" sheetId="3" r:id="Rbd5b4ee10eb64d5d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="쿠팡_일별입력" sheetId="4" r:id="Rb3602bdd34b94bf2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="일정표" sheetId="5" r:id="Rc5d2f1a0950f465d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="인사이트_액션플랜" sheetId="6" r:id="Rf329d8209e674322"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="운영_대시보드" sheetId="7" r:id="R209a72c74d7c4a28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="공개규칙" sheetId="8" r:id="R1a14563a21dc4e88"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -542,13 +541,13 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B7" s="21" t="str">
-        <x:v>보고서_목록 / 일정표</x:v>
+        <x:v>일정표</x:v>
       </x:c>
       <x:c r="C7" s="21" t="str">
-        <x:v>운영팀이 공개할 보고서, 일정, 요청사항을 정리합니다.</x:v>
+        <x:v>운영팀이 광고주 공유 로드맵과 일정, 요청사항을 직접 작성합니다.</x:v>
       </x:c>
       <x:c r="D7" s="21" t="str">
-        <x:v>필수 확인</x:v>
+        <x:v>운영팀 작성</x:v>
       </x:c>
       <x:c r="E7" s="21" t="str"/>
       <x:c r="F7" s="21" t="str"/>
@@ -563,10 +562,10 @@
         <x:v>인사이트_액션플랜</x:v>
       </x:c>
       <x:c r="C8" s="21" t="str">
-        <x:v>광고주에게 보여줄 결론과 다음 행동을 작성합니다.</x:v>
+        <x:v>운영팀이 광고주에게 보여줄 결론과 다음 행동을 직접 작성합니다.</x:v>
       </x:c>
       <x:c r="D8" s="21" t="str">
-        <x:v>짧게 작성</x:v>
+        <x:v>운영팀 작성</x:v>
       </x:c>
       <x:c r="E8" s="21" t="str"/>
       <x:c r="F8" s="21" t="str"/>
@@ -2937,426 +2936,6 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="13.329999923706055" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="13.329999923706055" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="34.439998626708984" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="12.220000267028809" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="11.109999656677246" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="12.4399995803833" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="33.33000183105469" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="25.5" customHeight="1">
-      <x:c r="A1" s="4" t="str">
-        <x:v>보고서 목록</x:v>
-      </x:c>
-      <x:c r="B1" s="4" t="str"/>
-      <x:c r="C1" s="4" t="str"/>
-      <x:c r="D1" s="4" t="str"/>
-      <x:c r="E1" s="4" t="str"/>
-      <x:c r="F1" s="4" t="str"/>
-      <x:c r="G1" s="4" t="str"/>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="13" t="str">
-        <x:v>운영팀이 공개할 보고서 파일명이나 링크를 정리합니다.</x:v>
-      </x:c>
-      <x:c r="B3" s="14" t="str"/>
-      <x:c r="C3" s="14" t="str"/>
-      <x:c r="D3" s="14" t="str"/>
-      <x:c r="E3" s="14" t="str"/>
-      <x:c r="F3" s="14" t="str"/>
-      <x:c r="G3" s="15" t="str"/>
-    </x:row>
-    <x:row r="5" ht="19.5" customHeight="1">
-      <x:c r="A5" s="26" t="str">
-        <x:v>보고서유형</x:v>
-      </x:c>
-      <x:c r="B5" s="26" t="str">
-        <x:v>기준기간</x:v>
-      </x:c>
-      <x:c r="C5" s="26" t="str">
-        <x:v>파일명/링크</x:v>
-      </x:c>
-      <x:c r="D5" s="26" t="str">
-        <x:v>공개상태</x:v>
-      </x:c>
-      <x:c r="E5" s="26" t="str">
-        <x:v>작성자</x:v>
-      </x:c>
-      <x:c r="F5" s="26" t="str">
-        <x:v>업데이트일</x:v>
-      </x:c>
-      <x:c r="G5" s="26" t="str">
-        <x:v>메모</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="19.5" customHeight="1">
-      <x:c r="A6" s="27" t="str">
-        <x:v>주간 보고서</x:v>
-      </x:c>
-      <x:c r="B6" s="27" t="str">
-        <x:v>2026-06 4주차</x:v>
-      </x:c>
-      <x:c r="C6" s="27" t="str">
-        <x:v>moment-weekly-202606-4.pdf</x:v>
-      </x:c>
-      <x:c r="D6" s="27" t="str">
-        <x:v>공개 가능</x:v>
-      </x:c>
-      <x:c r="E6" s="27" t="str">
-        <x:v>운영팀</x:v>
-      </x:c>
-      <x:c r="F6" s="27" t="str">
-        <x:v>2026-06-27</x:v>
-      </x:c>
-      <x:c r="G6" s="27" t="str">
-        <x:v>내부 메모 제거 후 공개</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="19.5" customHeight="1">
-      <x:c r="A7" s="27" t="str">
-        <x:v>월간 보고서</x:v>
-      </x:c>
-      <x:c r="B7" s="27" t="str">
-        <x:v>2026-06</x:v>
-      </x:c>
-      <x:c r="C7" s="27" t="str">
-        <x:v>moment-monthly-202606.pdf</x:v>
-      </x:c>
-      <x:c r="D7" s="27" t="str">
-        <x:v>검수 중</x:v>
-      </x:c>
-      <x:c r="E7" s="27" t="str">
-        <x:v>운영팀</x:v>
-      </x:c>
-      <x:c r="F7" s="27" t="str">
-        <x:v>2026-06-27</x:v>
-      </x:c>
-      <x:c r="G7" s="27" t="str">
-        <x:v>매출 수치 재확인</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="19.5" customHeight="1">
-      <x:c r="A8" s="27" t="str">
-        <x:v>KPI 보고서</x:v>
-      </x:c>
-      <x:c r="B8" s="27" t="str">
-        <x:v>2026-06</x:v>
-      </x:c>
-      <x:c r="C8" s="27" t="str">
-        <x:v>moment-kpi-202606.xlsx</x:v>
-      </x:c>
-      <x:c r="D8" s="27" t="str">
-        <x:v>공개 가능</x:v>
-      </x:c>
-      <x:c r="E8" s="27" t="str">
-        <x:v>운영팀</x:v>
-      </x:c>
-      <x:c r="F8" s="27" t="str">
-        <x:v>2026-06-27</x:v>
-      </x:c>
-      <x:c r="G8" s="27" t="str">
-        <x:v>목표달성률 포함</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="19.5" customHeight="1">
-      <x:c r="A9" s="27" t="str"/>
-      <x:c r="B9" s="27" t="str"/>
-      <x:c r="C9" s="27" t="str"/>
-      <x:c r="D9" s="27" t="str"/>
-      <x:c r="E9" s="27" t="str"/>
-      <x:c r="F9" s="27" t="str"/>
-      <x:c r="G9" s="27" t="str"/>
-    </x:row>
-    <x:row r="10" ht="19.5" customHeight="1">
-      <x:c r="A10" s="27"/>
-      <x:c r="B10" s="27"/>
-      <x:c r="C10" s="27"/>
-      <x:c r="D10" s="27"/>
-      <x:c r="E10" s="27"/>
-      <x:c r="F10" s="27"/>
-      <x:c r="G10" s="27"/>
-    </x:row>
-    <x:row r="11" ht="19.5" customHeight="1">
-      <x:c r="A11" s="27"/>
-      <x:c r="B11" s="27"/>
-      <x:c r="C11" s="27"/>
-      <x:c r="D11" s="27"/>
-      <x:c r="E11" s="27"/>
-      <x:c r="F11" s="27"/>
-      <x:c r="G11" s="27"/>
-    </x:row>
-    <x:row r="12" ht="19.5" customHeight="1">
-      <x:c r="A12" s="27"/>
-      <x:c r="B12" s="27"/>
-      <x:c r="C12" s="27"/>
-      <x:c r="D12" s="27"/>
-      <x:c r="E12" s="27"/>
-      <x:c r="F12" s="27"/>
-      <x:c r="G12" s="27"/>
-    </x:row>
-    <x:row r="13" ht="19.5" customHeight="1">
-      <x:c r="A13" s="27"/>
-      <x:c r="B13" s="27"/>
-      <x:c r="C13" s="27"/>
-      <x:c r="D13" s="27"/>
-      <x:c r="E13" s="27"/>
-      <x:c r="F13" s="27"/>
-      <x:c r="G13" s="27"/>
-    </x:row>
-    <x:row r="14" ht="19.5" customHeight="1">
-      <x:c r="A14" s="27"/>
-      <x:c r="B14" s="27"/>
-      <x:c r="C14" s="27"/>
-      <x:c r="D14" s="27"/>
-      <x:c r="E14" s="27"/>
-      <x:c r="F14" s="27"/>
-      <x:c r="G14" s="27"/>
-    </x:row>
-    <x:row r="15" ht="19.5" customHeight="1">
-      <x:c r="A15" s="27"/>
-      <x:c r="B15" s="27"/>
-      <x:c r="C15" s="27"/>
-      <x:c r="D15" s="27"/>
-      <x:c r="E15" s="27"/>
-      <x:c r="F15" s="27"/>
-      <x:c r="G15" s="27"/>
-    </x:row>
-    <x:row r="16" ht="19.5" customHeight="1">
-      <x:c r="A16" s="27"/>
-      <x:c r="B16" s="27"/>
-      <x:c r="C16" s="27"/>
-      <x:c r="D16" s="27"/>
-      <x:c r="E16" s="27"/>
-      <x:c r="F16" s="27"/>
-      <x:c r="G16" s="27"/>
-    </x:row>
-    <x:row r="17" ht="19.5" customHeight="1">
-      <x:c r="A17" s="27"/>
-      <x:c r="B17" s="27"/>
-      <x:c r="C17" s="27"/>
-      <x:c r="D17" s="27"/>
-      <x:c r="E17" s="27"/>
-      <x:c r="F17" s="27"/>
-      <x:c r="G17" s="27"/>
-    </x:row>
-    <x:row r="18" ht="19.5" customHeight="1">
-      <x:c r="A18" s="27"/>
-      <x:c r="B18" s="27"/>
-      <x:c r="C18" s="27"/>
-      <x:c r="D18" s="27"/>
-      <x:c r="E18" s="27"/>
-      <x:c r="F18" s="27"/>
-      <x:c r="G18" s="27"/>
-    </x:row>
-    <x:row r="19" ht="19.5" customHeight="1">
-      <x:c r="A19" s="27"/>
-      <x:c r="B19" s="27"/>
-      <x:c r="C19" s="27"/>
-      <x:c r="D19" s="27"/>
-      <x:c r="E19" s="27"/>
-      <x:c r="F19" s="27"/>
-      <x:c r="G19" s="27"/>
-    </x:row>
-    <x:row r="20" ht="19.5" customHeight="1">
-      <x:c r="A20" s="27"/>
-      <x:c r="B20" s="27"/>
-      <x:c r="C20" s="27"/>
-      <x:c r="D20" s="27"/>
-      <x:c r="E20" s="27"/>
-      <x:c r="F20" s="27"/>
-      <x:c r="G20" s="27"/>
-    </x:row>
-    <x:row r="21" ht="19.5" customHeight="1">
-      <x:c r="A21" s="27"/>
-      <x:c r="B21" s="27"/>
-      <x:c r="C21" s="27"/>
-      <x:c r="D21" s="27"/>
-      <x:c r="E21" s="27"/>
-      <x:c r="F21" s="27"/>
-      <x:c r="G21" s="27"/>
-    </x:row>
-    <x:row r="22" ht="19.5" customHeight="1">
-      <x:c r="A22" s="27"/>
-      <x:c r="B22" s="27"/>
-      <x:c r="C22" s="27"/>
-      <x:c r="D22" s="27"/>
-      <x:c r="E22" s="27"/>
-      <x:c r="F22" s="27"/>
-      <x:c r="G22" s="27"/>
-    </x:row>
-    <x:row r="23" ht="19.5" customHeight="1">
-      <x:c r="A23" s="27"/>
-      <x:c r="B23" s="27"/>
-      <x:c r="C23" s="27"/>
-      <x:c r="D23" s="27"/>
-      <x:c r="E23" s="27"/>
-      <x:c r="F23" s="27"/>
-      <x:c r="G23" s="27"/>
-    </x:row>
-    <x:row r="24" ht="19.5" customHeight="1">
-      <x:c r="A24" s="27"/>
-      <x:c r="B24" s="27"/>
-      <x:c r="C24" s="27"/>
-      <x:c r="D24" s="27"/>
-      <x:c r="E24" s="27"/>
-      <x:c r="F24" s="27"/>
-      <x:c r="G24" s="27"/>
-    </x:row>
-    <x:row r="25" ht="19.5" customHeight="1">
-      <x:c r="A25" s="27"/>
-      <x:c r="B25" s="27"/>
-      <x:c r="C25" s="27"/>
-      <x:c r="D25" s="27"/>
-      <x:c r="E25" s="27"/>
-      <x:c r="F25" s="27"/>
-      <x:c r="G25" s="27"/>
-    </x:row>
-    <x:row r="26" ht="19.5" customHeight="1">
-      <x:c r="A26" s="27"/>
-      <x:c r="B26" s="27"/>
-      <x:c r="C26" s="27"/>
-      <x:c r="D26" s="27"/>
-      <x:c r="E26" s="27"/>
-      <x:c r="F26" s="27"/>
-      <x:c r="G26" s="27"/>
-    </x:row>
-    <x:row r="27" ht="19.5" customHeight="1">
-      <x:c r="A27" s="27"/>
-      <x:c r="B27" s="27"/>
-      <x:c r="C27" s="27"/>
-      <x:c r="D27" s="27"/>
-      <x:c r="E27" s="27"/>
-      <x:c r="F27" s="27"/>
-      <x:c r="G27" s="27"/>
-    </x:row>
-    <x:row r="28" ht="19.5" customHeight="1">
-      <x:c r="A28" s="27"/>
-      <x:c r="B28" s="27"/>
-      <x:c r="C28" s="27"/>
-      <x:c r="D28" s="27"/>
-      <x:c r="E28" s="27"/>
-      <x:c r="F28" s="27"/>
-      <x:c r="G28" s="27"/>
-    </x:row>
-    <x:row r="29" ht="19.5" customHeight="1">
-      <x:c r="A29" s="27"/>
-      <x:c r="B29" s="27"/>
-      <x:c r="C29" s="27"/>
-      <x:c r="D29" s="27"/>
-      <x:c r="E29" s="27"/>
-      <x:c r="F29" s="27"/>
-      <x:c r="G29" s="27"/>
-    </x:row>
-    <x:row r="30" ht="19.5" customHeight="1">
-      <x:c r="A30" s="27"/>
-      <x:c r="B30" s="27"/>
-      <x:c r="C30" s="27"/>
-      <x:c r="D30" s="27"/>
-      <x:c r="E30" s="27"/>
-      <x:c r="F30" s="27"/>
-      <x:c r="G30" s="27"/>
-    </x:row>
-    <x:row r="31" ht="19.5" customHeight="1">
-      <x:c r="A31" s="27"/>
-      <x:c r="B31" s="27"/>
-      <x:c r="C31" s="27"/>
-      <x:c r="D31" s="27"/>
-      <x:c r="E31" s="27"/>
-      <x:c r="F31" s="27"/>
-      <x:c r="G31" s="27"/>
-    </x:row>
-    <x:row r="32" ht="19.5" customHeight="1">
-      <x:c r="A32" s="27"/>
-      <x:c r="B32" s="27"/>
-      <x:c r="C32" s="27"/>
-      <x:c r="D32" s="27"/>
-      <x:c r="E32" s="27"/>
-      <x:c r="F32" s="27"/>
-      <x:c r="G32" s="27"/>
-    </x:row>
-    <x:row r="33" ht="19.5" customHeight="1">
-      <x:c r="A33" s="27"/>
-      <x:c r="B33" s="27"/>
-      <x:c r="C33" s="27"/>
-      <x:c r="D33" s="27"/>
-      <x:c r="E33" s="27"/>
-      <x:c r="F33" s="27"/>
-      <x:c r="G33" s="27"/>
-    </x:row>
-    <x:row r="34" ht="19.5" customHeight="1">
-      <x:c r="A34" s="27"/>
-      <x:c r="B34" s="27"/>
-      <x:c r="C34" s="27"/>
-      <x:c r="D34" s="27"/>
-      <x:c r="E34" s="27"/>
-      <x:c r="F34" s="27"/>
-      <x:c r="G34" s="27"/>
-    </x:row>
-    <x:row r="35" ht="19.5" customHeight="1">
-      <x:c r="A35" s="27"/>
-      <x:c r="B35" s="27"/>
-      <x:c r="C35" s="27"/>
-      <x:c r="D35" s="27"/>
-      <x:c r="E35" s="27"/>
-      <x:c r="F35" s="27"/>
-      <x:c r="G35" s="27"/>
-    </x:row>
-    <x:row r="36" ht="19.5" customHeight="1">
-      <x:c r="A36" s="27"/>
-      <x:c r="B36" s="27"/>
-      <x:c r="C36" s="27"/>
-      <x:c r="D36" s="27"/>
-      <x:c r="E36" s="27"/>
-      <x:c r="F36" s="27"/>
-      <x:c r="G36" s="27"/>
-    </x:row>
-    <x:row r="37" ht="19.5" customHeight="1">
-      <x:c r="A37" s="27"/>
-      <x:c r="B37" s="27"/>
-      <x:c r="C37" s="27"/>
-      <x:c r="D37" s="27"/>
-      <x:c r="E37" s="27"/>
-      <x:c r="F37" s="27"/>
-      <x:c r="G37" s="27"/>
-    </x:row>
-    <x:row r="38" ht="19.5" customHeight="1">
-      <x:c r="A38" s="27"/>
-      <x:c r="B38" s="27"/>
-      <x:c r="C38" s="27"/>
-      <x:c r="D38" s="27"/>
-      <x:c r="E38" s="27"/>
-      <x:c r="F38" s="27"/>
-      <x:c r="G38" s="27"/>
-    </x:row>
-    <x:row r="39" ht="19.5" customHeight="1">
-      <x:c r="A39" s="27"/>
-      <x:c r="B39" s="27"/>
-      <x:c r="C39" s="27"/>
-      <x:c r="D39" s="27"/>
-      <x:c r="E39" s="27"/>
-      <x:c r="F39" s="27"/>
-      <x:c r="G39" s="27"/>
-    </x:row>
-    <x:row r="40" ht="19.5" customHeight="1">
-      <x:c r="A40" s="27"/>
-      <x:c r="B40" s="27"/>
-      <x:c r="C40" s="27"/>
-      <x:c r="D40" s="27"/>
-      <x:c r="E40" s="27"/>
-      <x:c r="F40" s="27"/>
-      <x:c r="G40" s="27"/>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
     <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="10" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="21.110000610351562" hidden="0" customWidth="1"/>
@@ -3381,7 +2960,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="13" t="str">
-        <x:v>광고주와 공유할 일정만 정리합니다. 내부 할 일은 메모에 구분해서 작성합니다.</x:v>
+        <x:v>운영팀이 광고주와 공유할 로드맵과 일정을 직접 작성합니다. 내부 할 일은 메모에 구분해서 작성합니다.</x:v>
       </x:c>
       <x:c r="B3" s="14" t="str"/>
       <x:c r="C3" s="14" t="str"/>
@@ -3870,7 +3449,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -4371,7 +3950,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -4561,12 +4140,12 @@
         <x:v>보고서 상태</x:v>
       </x:c>
       <x:c r="B11" s="28" t="str">
-        <x:f>IF(COUNTIF('보고서_목록'!D6:D40,"공개 가능")&gt;=1,"공개 가능","검수 필요")</x:f>
-        <x:v>공개 가능</x:v>
+        <x:f>IF(COUNTA('일정표'!A6:A40)+COUNTA('인사이트_액션플랜'!A6:A40)&gt;0,"작성 확인","작성 필요")</x:f>
+        <x:v>작성 확인</x:v>
       </x:c>
       <x:c r="C11" s="28" t="str">
         <x:f>B11</x:f>
-        <x:v>공개 가능</x:v>
+        <x:v>작성 확인</x:v>
       </x:c>
       <x:c r="D11" s="21"/>
       <x:c r="E11" s="21"/>
@@ -4638,10 +4217,10 @@
         <x:v>검수 중</x:v>
       </x:c>
       <x:c r="C16" s="21" t="str">
-        <x:v>파일 업로드</x:v>
+        <x:v>PPTX 생성</x:v>
       </x:c>
       <x:c r="D16" s="21" t="str">
-        <x:v>공개 가능 보고서만 광고주 노출</x:v>
+        <x:v>운영팀 작성값을 보고서 디자인에 배치</x:v>
       </x:c>
       <x:c r="E16" s="21"/>
       <x:c r="F16" s="21"/>
@@ -4709,7 +4288,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -4843,62 +4422,62 @@
     </x:row>
     <x:row r="10" ht="20.25" customHeight="1">
       <x:c r="A10" s="21" t="str">
-        <x:v>보고서_목록</x:v>
+        <x:v>일정표</x:v>
       </x:c>
       <x:c r="B10" s="21" t="str">
-        <x:v>보고서 파일명 또는 링크</x:v>
+        <x:v>광고주 공유 로드맵과 일정</x:v>
       </x:c>
       <x:c r="C10" s="21" t="str">
-        <x:v>공개 가능 상태만 노출</x:v>
+        <x:v>공개여부 Y만 노출</x:v>
       </x:c>
       <x:c r="D10" s="21" t="str">
-        <x:v>운영팀 작성</x:v>
+        <x:v>운영팀 직접 작성</x:v>
       </x:c>
       <x:c r="E10" s="21" t="str">
-        <x:v>필수</x:v>
+        <x:v>권장</x:v>
       </x:c>
       <x:c r="F10" s="21" t="str">
-        <x:v>업로드 후 확인</x:v>
+        <x:v>내부 일정은 N</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="20.25" customHeight="1">
       <x:c r="A11" s="21" t="str">
-        <x:v>일정표</x:v>
+        <x:v>인사이트</x:v>
       </x:c>
       <x:c r="B11" s="21" t="str">
-        <x:v>광고주 공유 일정</x:v>
+        <x:v>이번 주 결론과 다음 액션</x:v>
       </x:c>
       <x:c r="C11" s="21" t="str">
-        <x:v>공개여부 Y만 노출</x:v>
+        <x:v>공개코멘트만 노출</x:v>
       </x:c>
       <x:c r="D11" s="21" t="str">
-        <x:v>운영팀 작성</x:v>
+        <x:v>운영팀 직접 작성</x:v>
       </x:c>
       <x:c r="E11" s="21" t="str">
         <x:v>권장</x:v>
       </x:c>
       <x:c r="F11" s="21" t="str">
-        <x:v>내부 일정은 N</x:v>
+        <x:v>내부메모는 미노출</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="20.25" customHeight="1">
       <x:c r="A12" s="21" t="str">
-        <x:v>인사이트</x:v>
+        <x:v>PPTX 보고서</x:v>
       </x:c>
       <x:c r="B12" s="21" t="str">
-        <x:v>이번 주 결론과 다음 액션</x:v>
+        <x:v>웹 보고서함에서 생성되는 산출물</x:v>
       </x:c>
       <x:c r="C12" s="21" t="str">
-        <x:v>공개코멘트만 노출</x:v>
+        <x:v>검수 후 공개 파일만 노출</x:v>
       </x:c>
       <x:c r="D12" s="21" t="str">
-        <x:v>운영팀 작성</x:v>
+        <x:v>웹에서 생성·관리</x:v>
       </x:c>
       <x:c r="E12" s="21" t="str">
         <x:v>권장</x:v>
       </x:c>
       <x:c r="F12" s="21" t="str">
-        <x:v>내부메모는 미노출</x:v>
+        <x:v>엑셀 입력 시트 아님</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="20.25" customHeight="1">

</xml_diff>